<commit_message>
feat: close Wave 2 revised offer gate
</commit_message>
<xml_diff>
--- a/outputs/full-aura-audit/wave2-tender-pricing-proof.xlsx
+++ b/outputs/full-aura-audit/wave2-tender-pricing-proof.xlsx
@@ -429,7 +429,7 @@
         <v>Tender</v>
       </c>
       <c r="B3" t="str">
-        <v>Wave 2 governed CCTV Tender r1daco4</v>
+        <v>Wave 2 governed CCTV Tender r1mgoli</v>
       </c>
     </row>
     <row r="4">
@@ -437,7 +437,7 @@
         <v>Tender ID</v>
       </c>
       <c r="B4" t="str">
-        <v>a94bf63d-75ae-4ce1-af80-d9d88fad9e00</v>
+        <v>064942ff-eb92-4350-9034-7f23f51c8fd9</v>
       </c>
     </row>
     <row r="5">
@@ -445,7 +445,7 @@
         <v>Tender reference</v>
       </c>
       <c r="B5" t="str">
-        <v>W2-TDR-1789397954165</v>
+        <v>W2-TDR-1789413291024</v>
       </c>
     </row>
     <row r="6">
@@ -485,7 +485,7 @@
         <v>Technical Study ID</v>
       </c>
       <c r="B10" t="str">
-        <v>a4785a45-4c8d-4b08-8a0d-14786ae4a2b6</v>
+        <v>8ad9559a-fb6e-4236-bcfe-a37885bc3427</v>
       </c>
     </row>
     <row r="11">
@@ -509,7 +509,7 @@
         <v>BOQ ID</v>
       </c>
       <c r="B13" t="str">
-        <v>a8ea68e5-3514-409f-b1df-66581dfa9f38</v>
+        <v>c51ca5c2-4fdd-4948-a23d-67e8b4cac0fa</v>
       </c>
     </row>
     <row r="14">
@@ -517,7 +517,7 @@
         <v>Approved Quantity Take-Off ID</v>
       </c>
       <c r="B14" t="str">
-        <v>26d28f1b-e127-46b8-8933-2d51f9e6c489</v>
+        <v>f3115777-7554-4a4e-b174-ac22980bbb21</v>
       </c>
     </row>
     <row r="15">
@@ -533,7 +533,7 @@
         <v>Quantity projection time</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-09-14T14:59:15.702Z</v>
+        <v>2026-09-14T19:14:51.601Z</v>
       </c>
     </row>
     <row r="17">
@@ -829,13 +829,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>fafd0651-cb92-479a-af86-9b8f1d53df20</v>
+        <v>da0b6faf-c847-48ee-a8fa-9f2f5af7b340</v>
       </c>
       <c r="B2" t="str">
-        <v>468c6d19-238e-44a1-95ff-8b689cda78db</v>
+        <v>ddbb5116-4724-409c-8513-ac4aa3195f4c</v>
       </c>
       <c r="C2" t="str">
-        <v>a4785a45-4c8d-4b08-8a0d-14786ae4a2b6</v>
+        <v>8ad9559a-fb6e-4236-bcfe-a37885bc3427</v>
       </c>
       <c r="D2">
         <v>1</v>

</xml_diff>